<commit_message>
Changes on the project!
</commit_message>
<xml_diff>
--- a/util/Validation/ManualValidation/longParameterListForManual.xlsx
+++ b/util/Validation/ManualValidation/longParameterListForManual.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10111"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/neda/git/Research/BadSmells/util/Validation/ManualValidation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/neda/Desktop/workspace/BadSmells/util/Validation/ManualValidation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE5B7D80-6F14-C443-8713-88CBAB1A7FAC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5171B964-31FA-C046-88FE-7AFE6CC2207F}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="460" windowWidth="17560" windowHeight="14320" xr2:uid="{DD68CF97-1D9A-CC4B-9E29-4449E8DB2E7A}"/>
+    <workbookView xWindow="140" yWindow="460" windowWidth="17560" windowHeight="14260" xr2:uid="{DD68CF97-1D9A-CC4B-9E29-4449E8DB2E7A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -7195,10 +7195,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7517,17 +7518,17 @@
   <dimension ref="A1:G2372"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="32.33203125" customWidth="1"/>
+    <col min="1" max="1" width="32.33203125" style="3" customWidth="1"/>
     <col min="2" max="2" width="9" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="20.1640625" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" customWidth="1"/>
+    <col min="4" max="4" width="19.1640625" customWidth="1"/>
     <col min="5" max="5" width="12.6640625" customWidth="1"/>
     <col min="6" max="6" width="19.5" customWidth="1"/>
     <col min="7" max="7" width="63.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -8100,6 +8101,7 @@
       </c>
     </row>
     <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A24"/>
       <c r="F24" t="str">
         <f t="shared" si="1"/>
         <v>No</v>
@@ -8209,6 +8211,7 @@
       </c>
     </row>
     <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A29"/>
       <c r="F29" t="str">
         <f t="shared" si="1"/>
         <v>No</v>
@@ -8218,6 +8221,7 @@
       </c>
     </row>
     <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A30"/>
       <c r="F30" t="str">
         <f t="shared" si="1"/>
         <v>No</v>
@@ -8227,6 +8231,7 @@
       </c>
     </row>
     <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A31"/>
       <c r="F31" t="str">
         <f t="shared" si="1"/>
         <v>No</v>
@@ -8436,7 +8441,7 @@
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
+      <c r="A40" s="3" t="s">
         <v>50</v>
       </c>
       <c r="B40">
@@ -8486,6 +8491,7 @@
       </c>
     </row>
     <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A42"/>
       <c r="F42" t="str">
         <f t="shared" si="1"/>
         <v>No</v>
@@ -8495,6 +8501,7 @@
       </c>
     </row>
     <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A43"/>
       <c r="F43" t="str">
         <f t="shared" si="1"/>
         <v>No</v>
@@ -8504,6 +8511,7 @@
       </c>
     </row>
     <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A44"/>
       <c r="F44" t="str">
         <f t="shared" si="1"/>
         <v>No</v>
@@ -8513,6 +8521,7 @@
       </c>
     </row>
     <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A45"/>
       <c r="F45" t="str">
         <f t="shared" si="1"/>
         <v>No</v>
@@ -8522,6 +8531,7 @@
       </c>
     </row>
     <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A46"/>
       <c r="F46" t="str">
         <f t="shared" si="1"/>
         <v>No</v>
@@ -8531,6 +8541,7 @@
       </c>
     </row>
     <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A47"/>
       <c r="F47" t="str">
         <f t="shared" si="1"/>
         <v>No</v>
@@ -8540,6 +8551,7 @@
       </c>
     </row>
     <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A48"/>
       <c r="F48" t="str">
         <f t="shared" si="1"/>
         <v>No</v>
@@ -8699,6 +8711,7 @@
       </c>
     </row>
     <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A55"/>
       <c r="F55" t="str">
         <f t="shared" si="1"/>
         <v>No</v>
@@ -8708,6 +8721,7 @@
       </c>
     </row>
     <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A56"/>
       <c r="F56" t="str">
         <f t="shared" si="1"/>
         <v>No</v>
@@ -8717,6 +8731,7 @@
       </c>
     </row>
     <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A57"/>
       <c r="F57" t="str">
         <f t="shared" si="1"/>
         <v>No</v>
@@ -8726,6 +8741,7 @@
       </c>
     </row>
     <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A58"/>
       <c r="F58" t="str">
         <f t="shared" si="1"/>
         <v>No</v>
@@ -8735,6 +8751,7 @@
       </c>
     </row>
     <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A59"/>
       <c r="F59" t="str">
         <f t="shared" si="1"/>
         <v>No</v>
@@ -8744,6 +8761,7 @@
       </c>
     </row>
     <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A60"/>
       <c r="F60" t="str">
         <f t="shared" si="1"/>
         <v>No</v>
@@ -9253,6 +9271,7 @@
       </c>
     </row>
     <row r="81" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A81"/>
       <c r="E81" t="str">
         <f t="shared" si="5"/>
         <v>No</v>
@@ -9266,6 +9285,7 @@
       </c>
     </row>
     <row r="82" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A82"/>
       <c r="E82" t="str">
         <f t="shared" si="5"/>
         <v>No</v>
@@ -9279,6 +9299,7 @@
       </c>
     </row>
     <row r="83" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A83"/>
       <c r="E83" t="str">
         <f t="shared" si="5"/>
         <v>No</v>
@@ -9292,6 +9313,7 @@
       </c>
     </row>
     <row r="84" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A84"/>
       <c r="E84" t="str">
         <f t="shared" si="5"/>
         <v>No</v>
@@ -9305,6 +9327,7 @@
       </c>
     </row>
     <row r="85" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A85"/>
       <c r="E85" t="str">
         <f t="shared" si="5"/>
         <v>No</v>
@@ -9443,6 +9466,7 @@
       </c>
     </row>
     <row r="91" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A91"/>
       <c r="F91" t="str">
         <f t="shared" si="7"/>
         <v>No</v>
@@ -9452,6 +9476,7 @@
       </c>
     </row>
     <row r="92" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A92"/>
       <c r="F92" t="str">
         <f t="shared" si="7"/>
         <v>No</v>
@@ -9561,6 +9586,7 @@
       </c>
     </row>
     <row r="97" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A97"/>
       <c r="F97" t="str">
         <f t="shared" si="7"/>
         <v>No</v>
@@ -9570,6 +9596,7 @@
       </c>
     </row>
     <row r="98" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A98"/>
       <c r="F98" t="str">
         <f t="shared" si="7"/>
         <v>No</v>
@@ -9579,6 +9606,7 @@
       </c>
     </row>
     <row r="99" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A99"/>
       <c r="F99" t="str">
         <f t="shared" si="7"/>
         <v>No</v>
@@ -9588,6 +9616,7 @@
       </c>
     </row>
     <row r="100" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A100"/>
       <c r="F100" t="str">
         <f t="shared" si="7"/>
         <v>No</v>
@@ -9597,6 +9626,7 @@
       </c>
     </row>
     <row r="101" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A101"/>
       <c r="F101" t="str">
         <f t="shared" si="7"/>
         <v>No</v>
@@ -9606,6 +9636,7 @@
       </c>
     </row>
     <row r="102" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A102"/>
       <c r="F102" t="str">
         <f t="shared" si="7"/>
         <v>No</v>
@@ -9615,6 +9646,7 @@
       </c>
     </row>
     <row r="103" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A103"/>
       <c r="F103" t="str">
         <f t="shared" si="7"/>
         <v>No</v>
@@ -9624,6 +9656,7 @@
       </c>
     </row>
     <row r="104" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A104"/>
       <c r="F104" t="str">
         <f t="shared" si="7"/>
         <v>No</v>
@@ -9633,6 +9666,7 @@
       </c>
     </row>
     <row r="105" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A105"/>
       <c r="F105" t="str">
         <f t="shared" si="7"/>
         <v>No</v>
@@ -10992,6 +11026,7 @@
       </c>
     </row>
     <row r="160" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A160"/>
       <c r="F160" t="str">
         <f t="shared" si="11"/>
         <v>No</v>
@@ -11001,6 +11036,7 @@
       </c>
     </row>
     <row r="161" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A161"/>
       <c r="F161" t="str">
         <f t="shared" si="11"/>
         <v>No</v>
@@ -11635,6 +11671,7 @@
       </c>
     </row>
     <row r="187" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A187"/>
       <c r="F187" t="str">
         <f>IF(NOT(ISBLANK(A187)),"Yes","No")</f>
         <v>No</v>
@@ -11794,6 +11831,7 @@
       </c>
     </row>
     <row r="194" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A194"/>
       <c r="F194" t="str">
         <f t="shared" si="16"/>
         <v>No</v>
@@ -11903,6 +11941,7 @@
       </c>
     </row>
     <row r="199" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A199"/>
       <c r="F199" t="str">
         <f t="shared" si="16"/>
         <v>No</v>
@@ -12787,6 +12826,7 @@
       </c>
     </row>
     <row r="235" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A235"/>
       <c r="F235" t="str">
         <f t="shared" si="16"/>
         <v>No</v>
@@ -13021,7 +13061,7 @@
       </c>
     </row>
     <row r="245" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A245" t="s">
+      <c r="A245" s="3" t="s">
         <v>270</v>
       </c>
       <c r="B245">
@@ -13421,6 +13461,7 @@
       </c>
     </row>
     <row r="261" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A261"/>
       <c r="F261" t="str">
         <f t="shared" si="19"/>
         <v>No</v>
@@ -13480,6 +13521,7 @@
       </c>
     </row>
     <row r="264" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A264"/>
       <c r="F264" t="str">
         <f t="shared" si="19"/>
         <v>No</v>
@@ -15764,7 +15806,7 @@
       </c>
     </row>
     <row r="356" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A356" s="2" t="s">
+      <c r="A356" s="3" t="s">
         <v>390</v>
       </c>
       <c r="B356">
@@ -16039,7 +16081,7 @@
       </c>
     </row>
     <row r="367" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A367" s="2" t="s">
+      <c r="A367" s="3" t="s">
         <v>401</v>
       </c>
       <c r="B367">
@@ -16464,6 +16506,7 @@
       </c>
     </row>
     <row r="384" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A384"/>
       <c r="F384" t="str">
         <f t="shared" si="21"/>
         <v>No</v>
@@ -21248,6 +21291,7 @@
       </c>
     </row>
     <row r="576" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A576"/>
       <c r="F576" t="str">
         <f t="shared" si="30"/>
         <v>No</v>
@@ -23007,7 +23051,7 @@
       </c>
     </row>
     <row r="647" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A647" t="s">
+      <c r="A647" s="3" t="s">
         <v>680</v>
       </c>
       <c r="B647">
@@ -25282,6 +25326,7 @@
       </c>
     </row>
     <row r="738" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A738"/>
       <c r="F738" t="str">
         <f t="shared" si="35"/>
         <v>No</v>
@@ -25291,6 +25336,7 @@
       </c>
     </row>
     <row r="739" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A739"/>
       <c r="F739" t="str">
         <f t="shared" si="35"/>
         <v>No</v>
@@ -25300,6 +25346,7 @@
       </c>
     </row>
     <row r="740" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A740"/>
       <c r="F740" t="str">
         <f t="shared" si="35"/>
         <v>No</v>
@@ -25984,6 +26031,7 @@
       </c>
     </row>
     <row r="768" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A768"/>
       <c r="F768" t="str">
         <f t="shared" si="35"/>
         <v>No</v>
@@ -26043,6 +26091,7 @@
       </c>
     </row>
     <row r="771" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A771"/>
       <c r="F771" t="str">
         <f t="shared" si="35"/>
         <v>No</v>
@@ -26077,6 +26126,7 @@
       </c>
     </row>
     <row r="773" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A773"/>
       <c r="F773" t="str">
         <f t="shared" si="35"/>
         <v>No</v>
@@ -27561,6 +27611,7 @@
       </c>
     </row>
     <row r="833" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A833"/>
       <c r="F833" t="str">
         <f t="shared" si="38"/>
         <v>No</v>
@@ -27870,6 +27921,7 @@
       </c>
     </row>
     <row r="846" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A846"/>
       <c r="F846" t="str">
         <f t="shared" si="40"/>
         <v>No</v>
@@ -30554,6 +30606,7 @@
       </c>
     </row>
     <row r="954" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A954"/>
       <c r="F954" t="str">
         <f t="shared" si="42"/>
         <v>No</v>
@@ -30563,6 +30616,7 @@
       </c>
     </row>
     <row r="955" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A955"/>
       <c r="F955" t="str">
         <f t="shared" si="42"/>
         <v>No</v>
@@ -30922,6 +30976,7 @@
       </c>
     </row>
     <row r="970" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A970"/>
       <c r="F970" t="str">
         <f t="shared" si="42"/>
         <v>No</v>
@@ -31081,6 +31136,7 @@
       </c>
     </row>
     <row r="977" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A977"/>
       <c r="F977" t="str">
         <f t="shared" si="44"/>
         <v>No</v>
@@ -31140,6 +31196,7 @@
       </c>
     </row>
     <row r="980" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A980"/>
       <c r="F980" t="str">
         <f t="shared" si="44"/>
         <v>No</v>
@@ -31149,6 +31206,7 @@
       </c>
     </row>
     <row r="981" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A981"/>
       <c r="F981" t="str">
         <f t="shared" si="44"/>
         <v>No</v>
@@ -31283,6 +31341,7 @@
       </c>
     </row>
     <row r="987" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A987"/>
       <c r="F987" t="str">
         <f t="shared" si="44"/>
         <v>No</v>
@@ -31317,6 +31376,7 @@
       </c>
     </row>
     <row r="989" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A989"/>
       <c r="F989" t="str">
         <f t="shared" si="44"/>
         <v>No</v>
@@ -31326,6 +31386,7 @@
       </c>
     </row>
     <row r="990" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A990"/>
       <c r="F990" t="str">
         <f t="shared" si="44"/>
         <v>No</v>
@@ -31335,6 +31396,7 @@
       </c>
     </row>
     <row r="991" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A991"/>
       <c r="F991" t="str">
         <f t="shared" si="44"/>
         <v>No</v>
@@ -31344,6 +31406,7 @@
       </c>
     </row>
     <row r="992" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A992"/>
       <c r="F992" t="str">
         <f t="shared" si="44"/>
         <v>No</v>
@@ -31353,6 +31416,7 @@
       </c>
     </row>
     <row r="993" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A993"/>
       <c r="F993" t="str">
         <f t="shared" si="44"/>
         <v>No</v>
@@ -31362,6 +31426,7 @@
       </c>
     </row>
     <row r="994" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A994"/>
       <c r="F994" t="str">
         <f t="shared" si="44"/>
         <v>No</v>
@@ -31371,6 +31436,7 @@
       </c>
     </row>
     <row r="995" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A995"/>
       <c r="F995" t="str">
         <f t="shared" si="44"/>
         <v>No</v>
@@ -31380,6 +31446,7 @@
       </c>
     </row>
     <row r="996" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A996"/>
       <c r="F996" t="str">
         <f t="shared" si="44"/>
         <v>No</v>
@@ -31814,6 +31881,7 @@
       </c>
     </row>
     <row r="1014" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1014"/>
       <c r="F1014" t="str">
         <f t="shared" si="44"/>
         <v>No</v>
@@ -31823,6 +31891,7 @@
       </c>
     </row>
     <row r="1015" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1015"/>
       <c r="E1015" t="str">
         <f t="shared" si="43"/>
         <v>No</v>
@@ -31836,6 +31905,7 @@
       </c>
     </row>
     <row r="1016" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1016"/>
       <c r="E1016" t="str">
         <f t="shared" si="43"/>
         <v>No</v>
@@ -31849,6 +31919,7 @@
       </c>
     </row>
     <row r="1017" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1017"/>
       <c r="E1017" t="str">
         <f t="shared" si="43"/>
         <v>No</v>
@@ -31912,6 +31983,7 @@
       </c>
     </row>
     <row r="1020" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1020"/>
       <c r="F1020" t="str">
         <f t="shared" ref="F1020:F1021" si="45">IF(NOT(ISBLANK(A1020)),"Yes","No")</f>
         <v>No</v>
@@ -31921,6 +31993,7 @@
       </c>
     </row>
     <row r="1021" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1021"/>
       <c r="F1021" t="str">
         <f t="shared" si="45"/>
         <v>No</v>
@@ -31955,6 +32028,7 @@
       </c>
     </row>
     <row r="1023" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1023"/>
       <c r="F1023" t="str">
         <f t="shared" si="47"/>
         <v>No</v>
@@ -31964,6 +32038,7 @@
       </c>
     </row>
     <row r="1024" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1024"/>
       <c r="F1024" t="str">
         <f t="shared" si="47"/>
         <v>No</v>
@@ -31973,6 +32048,7 @@
       </c>
     </row>
     <row r="1025" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1025"/>
       <c r="F1025" t="str">
         <f t="shared" si="47"/>
         <v>No</v>
@@ -31982,6 +32058,7 @@
       </c>
     </row>
     <row r="1026" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1026"/>
       <c r="F1026" t="str">
         <f t="shared" ref="F1026:F1032" si="48">IF(NOT(ISBLANK(A1026)),"Yes","No")</f>
         <v>No</v>
@@ -31991,6 +32068,7 @@
       </c>
     </row>
     <row r="1027" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1027"/>
       <c r="F1027" t="str">
         <f t="shared" si="48"/>
         <v>No</v>
@@ -32000,6 +32078,7 @@
       </c>
     </row>
     <row r="1028" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1028"/>
       <c r="F1028" t="str">
         <f t="shared" si="48"/>
         <v>No</v>
@@ -32009,6 +32088,7 @@
       </c>
     </row>
     <row r="1029" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1029"/>
       <c r="F1029" t="str">
         <f t="shared" si="48"/>
         <v>No</v>
@@ -32018,6 +32098,7 @@
       </c>
     </row>
     <row r="1030" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1030"/>
       <c r="F1030" t="str">
         <f t="shared" si="48"/>
         <v>No</v>
@@ -32027,6 +32108,7 @@
       </c>
     </row>
     <row r="1031" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1031"/>
       <c r="F1031" t="str">
         <f t="shared" si="48"/>
         <v>No</v>
@@ -32036,6 +32118,7 @@
       </c>
     </row>
     <row r="1032" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1032"/>
       <c r="F1032" t="str">
         <f t="shared" si="48"/>
         <v>No</v>
@@ -32045,6 +32128,7 @@
       </c>
     </row>
     <row r="1033" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1033"/>
       <c r="F1033" t="str">
         <f t="shared" ref="F1033:F1039" si="49">IF(NOT(ISBLANK(A1033)),"Yes","No")</f>
         <v>No</v>
@@ -32054,6 +32138,7 @@
       </c>
     </row>
     <row r="1034" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1034"/>
       <c r="F1034" t="str">
         <f t="shared" si="49"/>
         <v>No</v>
@@ -32063,6 +32148,7 @@
       </c>
     </row>
     <row r="1035" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1035"/>
       <c r="F1035" t="str">
         <f t="shared" si="49"/>
         <v>No</v>
@@ -32097,6 +32183,7 @@
       </c>
     </row>
     <row r="1037" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1037"/>
       <c r="F1037" t="str">
         <f t="shared" si="49"/>
         <v>No</v>
@@ -32106,6 +32193,7 @@
       </c>
     </row>
     <row r="1038" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1038"/>
       <c r="F1038" t="str">
         <f t="shared" si="49"/>
         <v>No</v>
@@ -32115,6 +32203,7 @@
       </c>
     </row>
     <row r="1039" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1039"/>
       <c r="F1039" t="str">
         <f t="shared" si="49"/>
         <v>No</v>
@@ -32124,6 +32213,7 @@
       </c>
     </row>
     <row r="1040" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1040"/>
       <c r="F1040" t="str">
         <f t="shared" ref="F1040:F1048" si="50">IF(NOT(ISBLANK(A1040)),"Yes","No")</f>
         <v>No</v>
@@ -32133,6 +32223,7 @@
       </c>
     </row>
     <row r="1041" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1041"/>
       <c r="F1041" t="str">
         <f t="shared" si="50"/>
         <v>No</v>
@@ -32142,6 +32233,7 @@
       </c>
     </row>
     <row r="1042" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1042"/>
       <c r="F1042" t="str">
         <f t="shared" si="50"/>
         <v>No</v>
@@ -32151,6 +32243,7 @@
       </c>
     </row>
     <row r="1043" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1043"/>
       <c r="F1043" t="str">
         <f t="shared" si="50"/>
         <v>No</v>
@@ -32160,6 +32253,7 @@
       </c>
     </row>
     <row r="1044" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1044"/>
       <c r="F1044" t="str">
         <f t="shared" si="50"/>
         <v>No</v>
@@ -32169,6 +32263,7 @@
       </c>
     </row>
     <row r="1045" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1045"/>
       <c r="F1045" t="str">
         <f t="shared" si="50"/>
         <v>No</v>
@@ -32203,6 +32298,7 @@
       </c>
     </row>
     <row r="1047" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1047"/>
       <c r="E1047" t="str">
         <f t="shared" si="46"/>
         <v>No</v>
@@ -32216,6 +32312,7 @@
       </c>
     </row>
     <row r="1048" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1048"/>
       <c r="E1048" t="str">
         <f t="shared" si="46"/>
         <v>No</v>
@@ -37304,6 +37401,7 @@
       </c>
     </row>
     <row r="1252" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1252"/>
       <c r="F1252" t="str">
         <f t="shared" ref="F1252:F1264" si="58">IF(NOT(ISBLANK(A1252)),"Yes","No")</f>
         <v>No</v>
@@ -37613,6 +37711,7 @@
       </c>
     </row>
     <row r="1265" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1265"/>
       <c r="F1265" t="str">
         <f t="shared" ref="F1265" si="60">IF(NOT(ISBLANK(A1265)),"Yes","No")</f>
         <v>No</v>
@@ -38322,6 +38421,7 @@
       </c>
     </row>
     <row r="1294" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1294"/>
       <c r="E1294" t="str">
         <f t="shared" si="63"/>
         <v>No</v>
@@ -38335,6 +38435,7 @@
       </c>
     </row>
     <row r="1295" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1295"/>
       <c r="E1295" t="str">
         <f t="shared" si="63"/>
         <v>No</v>
@@ -38373,7 +38474,7 @@
       </c>
     </row>
     <row r="1297" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1297" t="s">
+      <c r="A1297" s="2" t="s">
         <v>1329</v>
       </c>
       <c r="B1297">
@@ -38698,6 +38799,7 @@
       </c>
     </row>
     <row r="1310" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1310"/>
       <c r="F1310" t="str">
         <f t="shared" ref="F1310:F1323" si="69">IF(NOT(ISBLANK(A1310)),"Yes","No")</f>
         <v>No</v>
@@ -39132,7 +39234,7 @@
       </c>
     </row>
     <row r="1328" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1328" t="s">
+      <c r="A1328" s="3" t="s">
         <v>1361</v>
       </c>
       <c r="B1328">
@@ -39507,6 +39609,7 @@
       </c>
     </row>
     <row r="1343" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1343"/>
       <c r="F1343" t="str">
         <f t="shared" ref="F1343:F1386" si="73">IF(NOT(ISBLANK(A1343)),"Yes","No")</f>
         <v>No</v>
@@ -39541,7 +39644,7 @@
       </c>
     </row>
     <row r="1345" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1345" s="2" t="s">
+      <c r="A1345" s="3" t="s">
         <v>1379</v>
       </c>
       <c r="B1345">
@@ -39566,7 +39669,7 @@
       </c>
     </row>
     <row r="1346" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1346" s="2" t="s">
+      <c r="A1346" s="3" t="s">
         <v>1380</v>
       </c>
       <c r="B1346">
@@ -39591,7 +39694,7 @@
       </c>
     </row>
     <row r="1347" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1347" s="2" t="s">
+      <c r="A1347" s="3" t="s">
         <v>1381</v>
       </c>
       <c r="B1347">
@@ -39616,7 +39719,7 @@
       </c>
     </row>
     <row r="1348" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1348" s="2" t="s">
+      <c r="A1348" s="3" t="s">
         <v>1382</v>
       </c>
       <c r="B1348">
@@ -39641,7 +39744,7 @@
       </c>
     </row>
     <row r="1349" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1349" s="2" t="s">
+      <c r="A1349" s="3" t="s">
         <v>1383</v>
       </c>
       <c r="B1349">
@@ -39666,7 +39769,7 @@
       </c>
     </row>
     <row r="1350" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1350" s="2" t="s">
+      <c r="A1350" s="3" t="s">
         <v>1384</v>
       </c>
       <c r="B1350">
@@ -39691,7 +39794,7 @@
       </c>
     </row>
     <row r="1351" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1351" s="2" t="s">
+      <c r="A1351" s="3" t="s">
         <v>1385</v>
       </c>
       <c r="B1351">
@@ -39716,7 +39819,7 @@
       </c>
     </row>
     <row r="1352" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1352" s="2" t="s">
+      <c r="A1352" s="3" t="s">
         <v>1386</v>
       </c>
       <c r="B1352">
@@ -39741,7 +39844,7 @@
       </c>
     </row>
     <row r="1353" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1353" s="2" t="s">
+      <c r="A1353" s="3" t="s">
         <v>1387</v>
       </c>
       <c r="B1353">
@@ -39766,7 +39869,7 @@
       </c>
     </row>
     <row r="1354" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1354" s="2" t="s">
+      <c r="A1354" s="3" t="s">
         <v>1388</v>
       </c>
       <c r="B1354">
@@ -39791,7 +39894,7 @@
       </c>
     </row>
     <row r="1355" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1355" s="2" t="s">
+      <c r="A1355" s="3" t="s">
         <v>1389</v>
       </c>
       <c r="B1355">
@@ -39816,7 +39919,7 @@
       </c>
     </row>
     <row r="1356" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1356" s="2" t="s">
+      <c r="A1356" s="3" t="s">
         <v>1390</v>
       </c>
       <c r="B1356">
@@ -39841,7 +39944,7 @@
       </c>
     </row>
     <row r="1357" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1357" s="2" t="s">
+      <c r="A1357" s="3" t="s">
         <v>1391</v>
       </c>
       <c r="B1357">
@@ -39866,7 +39969,7 @@
       </c>
     </row>
     <row r="1358" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1358" s="2" t="s">
+      <c r="A1358" s="3" t="s">
         <v>1392</v>
       </c>
       <c r="B1358">
@@ -39891,7 +39994,7 @@
       </c>
     </row>
     <row r="1359" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1359" s="2" t="s">
+      <c r="A1359" s="3" t="s">
         <v>1393</v>
       </c>
       <c r="B1359">
@@ -39916,7 +40019,7 @@
       </c>
     </row>
     <row r="1360" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1360" s="2" t="s">
+      <c r="A1360" s="3" t="s">
         <v>1394</v>
       </c>
       <c r="B1360">
@@ -44416,7 +44519,7 @@
       </c>
     </row>
     <row r="1540" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1540" s="2" t="s">
+      <c r="A1540" s="3" t="s">
         <v>1581</v>
       </c>
       <c r="B1540">
@@ -44588,7 +44691,7 @@
       </c>
     </row>
     <row r="1547" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1547" t="s">
+      <c r="A1547" s="3" t="s">
         <v>1587</v>
       </c>
       <c r="B1547">
@@ -49163,6 +49266,7 @@
       </c>
     </row>
     <row r="1730" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1730"/>
       <c r="F1730" t="str">
         <f t="shared" ref="F1730:F1756" si="100">IF(NOT(ISBLANK(A1730)),"Yes","No")</f>
         <v>No</v>
@@ -49472,7 +49576,7 @@
       </c>
     </row>
     <row r="1743" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1743" t="s">
+      <c r="A1743" s="3" t="s">
         <v>1782</v>
       </c>
       <c r="B1743">
@@ -49647,6 +49751,7 @@
       </c>
     </row>
     <row r="1750" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1750"/>
       <c r="F1750" t="str">
         <f t="shared" si="100"/>
         <v>No</v>
@@ -49656,6 +49761,7 @@
       </c>
     </row>
     <row r="1751" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1751"/>
       <c r="F1751" t="str">
         <f t="shared" si="100"/>
         <v>No</v>
@@ -51090,7 +51196,7 @@
       </c>
     </row>
     <row r="1809" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1809" t="s">
+      <c r="A1809" s="3" t="s">
         <v>1847</v>
       </c>
       <c r="B1809">
@@ -52165,6 +52271,7 @@
       </c>
     </row>
     <row r="1852" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1852"/>
       <c r="F1852" t="str">
         <f t="shared" ref="F1852" si="108">IF(NOT(ISBLANK(A1852)),"Yes","No")</f>
         <v>No</v>
@@ -52174,6 +52281,7 @@
       </c>
     </row>
     <row r="1853" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A1853"/>
       <c r="F1853" t="str">
         <f t="shared" ref="F1853" si="109">IF(NOT(ISBLANK(A1853)),"Yes","No")</f>
         <v>No</v>
@@ -53583,7 +53691,7 @@
       </c>
     </row>
     <row r="1910" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1910" t="s">
+      <c r="A1910" s="3" t="s">
         <v>219</v>
       </c>
       <c r="B1910">
@@ -56008,6 +56116,7 @@
       </c>
     </row>
     <row r="2007" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2007"/>
       <c r="F2007" t="str">
         <f t="shared" ref="F2007:F2009" si="117">IF(NOT(ISBLANK(A2007)),"Yes","No")</f>
         <v>No</v>
@@ -56017,6 +56126,7 @@
       </c>
     </row>
     <row r="2008" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2008"/>
       <c r="F2008" t="str">
         <f t="shared" si="117"/>
         <v>No</v>
@@ -56026,6 +56136,7 @@
       </c>
     </row>
     <row r="2009" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2009"/>
       <c r="F2009" t="str">
         <f t="shared" si="117"/>
         <v>No</v>
@@ -56160,6 +56271,7 @@
       </c>
     </row>
     <row r="2015" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2015"/>
       <c r="F2015" t="str">
         <f t="shared" si="121"/>
         <v>No</v>
@@ -56344,7 +56456,7 @@
       </c>
     </row>
     <row r="2023" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2023" t="s">
+      <c r="A2023" s="3" t="s">
         <v>2017</v>
       </c>
       <c r="B2023">
@@ -56394,7 +56506,7 @@
       </c>
     </row>
     <row r="2025" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2025" t="s">
+      <c r="A2025" s="3" t="s">
         <v>2019</v>
       </c>
       <c r="B2025">
@@ -56594,7 +56706,7 @@
       </c>
     </row>
     <row r="2033" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2033" t="s">
+      <c r="A2033" s="3" t="s">
         <v>2027</v>
       </c>
       <c r="B2033">
@@ -61244,6 +61356,7 @@
       </c>
     </row>
     <row r="2219" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2219"/>
       <c r="F2219" t="str">
         <f t="shared" ref="F2219:F2225" si="131">IF(NOT(ISBLANK(A2219)),"Yes","No")</f>
         <v>No</v>
@@ -61378,6 +61491,7 @@
       </c>
     </row>
     <row r="2225" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2225"/>
       <c r="F2225" t="str">
         <f t="shared" si="131"/>
         <v>No</v>
@@ -61412,6 +61526,7 @@
       </c>
     </row>
     <row r="2227" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2227"/>
       <c r="F2227" t="str">
         <f t="shared" si="133"/>
         <v>No</v>
@@ -61571,6 +61686,7 @@
       </c>
     </row>
     <row r="2234" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2234"/>
       <c r="F2234" t="str">
         <f t="shared" ref="F2234:F2238" si="134">IF(NOT(ISBLANK(A2234)),"Yes","No")</f>
         <v>No</v>
@@ -61580,6 +61696,7 @@
       </c>
     </row>
     <row r="2235" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2235"/>
       <c r="F2235" t="str">
         <f t="shared" si="134"/>
         <v>No</v>
@@ -61589,6 +61706,7 @@
       </c>
     </row>
     <row r="2236" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2236"/>
       <c r="F2236" t="str">
         <f t="shared" si="134"/>
         <v>No</v>
@@ -61623,7 +61741,7 @@
       </c>
     </row>
     <row r="2238" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2238" t="s">
+      <c r="A2238" s="2" t="s">
         <v>2226</v>
       </c>
       <c r="B2238">
@@ -61673,6 +61791,7 @@
       </c>
     </row>
     <row r="2240" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2240"/>
       <c r="F2240" t="str">
         <f t="shared" si="137"/>
         <v>No</v>
@@ -61682,6 +61801,7 @@
       </c>
     </row>
     <row r="2241" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2241"/>
       <c r="E2241" t="str">
         <f t="shared" si="136"/>
         <v>No</v>
@@ -62070,6 +62190,7 @@
       </c>
     </row>
     <row r="2257" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2257"/>
       <c r="F2257" t="str">
         <f t="shared" ref="F2257:F2277" si="138">IF(NOT(ISBLANK(A2257)),"Yes","No")</f>
         <v>No</v>
@@ -62454,7 +62575,7 @@
       </c>
     </row>
     <row r="2273" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2273" t="s">
+      <c r="A2273" s="3" t="s">
         <v>2262</v>
       </c>
       <c r="B2273">
@@ -62704,7 +62825,7 @@
       </c>
     </row>
     <row r="2283" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2283" t="s">
+      <c r="A2283" s="3" t="s">
         <v>2273</v>
       </c>
       <c r="B2283">
@@ -62854,7 +62975,7 @@
       </c>
     </row>
     <row r="2289" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2289" t="s">
+      <c r="A2289" s="3" t="s">
         <v>2276</v>
       </c>
       <c r="B2289">
@@ -62929,7 +63050,7 @@
       </c>
     </row>
     <row r="2292" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2292" t="s">
+      <c r="A2292" s="3" t="s">
         <v>2279</v>
       </c>
       <c r="B2292">
@@ -63004,7 +63125,7 @@
       </c>
     </row>
     <row r="2295" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2295" t="s">
+      <c r="A2295" s="3" t="s">
         <v>2282</v>
       </c>
       <c r="B2295">
@@ -63129,7 +63250,7 @@
       </c>
     </row>
     <row r="2300" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2300" t="s">
+      <c r="A2300" s="3" t="s">
         <v>2287</v>
       </c>
       <c r="B2300">
@@ -63429,7 +63550,7 @@
       </c>
     </row>
     <row r="2312" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2312" t="s">
+      <c r="A2312" s="3" t="s">
         <v>2298</v>
       </c>
       <c r="B2312">
@@ -64104,6 +64225,7 @@
       </c>
     </row>
     <row r="2339" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2339"/>
       <c r="F2339" t="str">
         <f t="shared" ref="F2339:F2345" si="142">IF(NOT(ISBLANK(A2339)),"Yes","No")</f>
         <v>No</v>
@@ -64113,6 +64235,7 @@
       </c>
     </row>
     <row r="2340" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2340"/>
       <c r="F2340" t="str">
         <f t="shared" si="142"/>
         <v>No</v>
@@ -64147,6 +64270,7 @@
       </c>
     </row>
     <row r="2342" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2342"/>
       <c r="F2342" t="str">
         <f t="shared" si="142"/>
         <v>No</v>
@@ -64156,6 +64280,7 @@
       </c>
     </row>
     <row r="2343" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2343"/>
       <c r="F2343" t="str">
         <f t="shared" si="142"/>
         <v>No</v>
@@ -64165,6 +64290,7 @@
       </c>
     </row>
     <row r="2344" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2344"/>
       <c r="F2344" t="str">
         <f t="shared" si="142"/>
         <v>No</v>
@@ -64174,6 +64300,7 @@
       </c>
     </row>
     <row r="2345" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2345"/>
       <c r="F2345" t="str">
         <f t="shared" si="142"/>
         <v>No</v>
@@ -64183,6 +64310,7 @@
       </c>
     </row>
     <row r="2346" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2346"/>
       <c r="F2346" t="str">
         <f t="shared" ref="F2346:F2356" si="144">IF(NOT(ISBLANK(A2346)),"Yes","No")</f>
         <v>No</v>
@@ -64192,6 +64320,7 @@
       </c>
     </row>
     <row r="2347" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2347"/>
       <c r="F2347" t="str">
         <f t="shared" si="144"/>
         <v>No</v>
@@ -64201,6 +64330,7 @@
       </c>
     </row>
     <row r="2348" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2348"/>
       <c r="F2348" t="str">
         <f t="shared" si="144"/>
         <v>No</v>
@@ -64210,6 +64340,7 @@
       </c>
     </row>
     <row r="2349" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2349"/>
       <c r="F2349" t="str">
         <f t="shared" si="144"/>
         <v>No</v>
@@ -64219,6 +64350,7 @@
       </c>
     </row>
     <row r="2350" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2350"/>
       <c r="F2350" t="str">
         <f t="shared" si="144"/>
         <v>No</v>
@@ -64228,6 +64360,7 @@
       </c>
     </row>
     <row r="2351" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2351"/>
       <c r="F2351" t="str">
         <f t="shared" si="144"/>
         <v>No</v>
@@ -64237,6 +64370,7 @@
       </c>
     </row>
     <row r="2352" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2352"/>
       <c r="F2352" t="str">
         <f t="shared" si="144"/>
         <v>No</v>
@@ -64246,6 +64380,7 @@
       </c>
     </row>
     <row r="2353" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2353"/>
       <c r="F2353" t="str">
         <f t="shared" si="144"/>
         <v>No</v>
@@ -64255,6 +64390,7 @@
       </c>
     </row>
     <row r="2354" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2354"/>
       <c r="F2354" t="str">
         <f t="shared" si="144"/>
         <v>No</v>
@@ -64264,6 +64400,7 @@
       </c>
     </row>
     <row r="2355" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2355"/>
       <c r="F2355" t="str">
         <f t="shared" si="144"/>
         <v>No</v>
@@ -64273,6 +64410,7 @@
       </c>
     </row>
     <row r="2356" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2356"/>
       <c r="F2356" t="str">
         <f t="shared" si="144"/>
         <v>No</v>
@@ -64282,6 +64420,7 @@
       </c>
     </row>
     <row r="2357" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2357"/>
       <c r="F2357" t="str">
         <f t="shared" ref="F2357:F2361" si="145">IF(NOT(ISBLANK(A2357)),"Yes","No")</f>
         <v>No</v>
@@ -64341,6 +64480,7 @@
       </c>
     </row>
     <row r="2360" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2360"/>
       <c r="F2360" t="str">
         <f t="shared" si="145"/>
         <v>No</v>
@@ -64350,6 +64490,7 @@
       </c>
     </row>
     <row r="2361" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2361"/>
       <c r="F2361" t="str">
         <f t="shared" si="145"/>
         <v>No</v>
@@ -64359,6 +64500,7 @@
       </c>
     </row>
     <row r="2362" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2362"/>
       <c r="F2362" t="str">
         <f t="shared" ref="F2362:F2366" si="147">IF(NOT(ISBLANK(A2362)),"Yes","No")</f>
         <v>No</v>
@@ -64368,6 +64510,7 @@
       </c>
     </row>
     <row r="2363" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2363"/>
       <c r="F2363" t="str">
         <f t="shared" si="147"/>
         <v>No</v>
@@ -64377,6 +64520,7 @@
       </c>
     </row>
     <row r="2364" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2364"/>
       <c r="F2364" t="str">
         <f t="shared" si="147"/>
         <v>No</v>
@@ -64386,6 +64530,7 @@
       </c>
     </row>
     <row r="2365" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2365"/>
       <c r="F2365" t="str">
         <f t="shared" si="147"/>
         <v>No</v>
@@ -64395,6 +64540,7 @@
       </c>
     </row>
     <row r="2366" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2366"/>
       <c r="F2366" t="str">
         <f t="shared" si="147"/>
         <v>No</v>
@@ -64404,6 +64550,7 @@
       </c>
     </row>
     <row r="2367" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2367"/>
       <c r="F2367" t="str">
         <f t="shared" ref="F2367:F2371" si="148">IF(NOT(ISBLANK(A2367)),"Yes","No")</f>
         <v>No</v>
@@ -64413,6 +64560,7 @@
       </c>
     </row>
     <row r="2368" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A2368"/>
       <c r="F2368" t="str">
         <f t="shared" si="148"/>
         <v>No</v>
@@ -64421,7 +64569,7 @@
         <v>2351</v>
       </c>
     </row>
-    <row r="2369" spans="6:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2369" spans="6:7" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
       <c r="F2369" t="str">
         <f t="shared" si="148"/>
         <v>No</v>
@@ -64430,7 +64578,7 @@
         <v>2352</v>
       </c>
     </row>
-    <row r="2370" spans="6:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2370" spans="6:7" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
       <c r="F2370" t="str">
         <f t="shared" si="148"/>
         <v>No</v>
@@ -64439,7 +64587,7 @@
         <v>2353</v>
       </c>
     </row>
-    <row r="2371" spans="6:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2371" spans="6:7" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
       <c r="F2371" t="str">
         <f t="shared" si="148"/>
         <v>No</v>
@@ -64448,7 +64596,7 @@
         <v>2354</v>
       </c>
     </row>
-    <row r="2372" spans="6:7" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2372" spans="6:7" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
       <c r="F2372" t="str">
         <f t="shared" ref="F2372" si="149">IF(NOT(ISBLANK(A2372)),"Yes","No")</f>
         <v>No</v>

</xml_diff>